<commit_message>
+ thong ke PN, down EPPlus -> ver 4.5.3.3
</commit_message>
<xml_diff>
--- a/DanhSachNhanVien.xlsx
+++ b/DanhSachNhanVien.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\CoffeeManagement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\CoffeeManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0659724E-146D-4FAC-B40F-841DB676BA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6054D2-9334-4133-BA7F-3BEF09EC8086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NhanVien" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -52,33 +52,36 @@
     <t>UserID</t>
   </si>
   <si>
-    <t>s</t>
+    <t>Nguyễn</t>
   </si>
   <si>
     <t>An</t>
   </si>
   <si>
-    <t>s An</t>
-  </si>
-  <si>
-    <t>0909000009</t>
-  </si>
-  <si>
-    <t>Đang làm</t>
-  </si>
-  <si>
-    <t>08/12/2025</t>
+    <t>Nguyễn An</t>
+  </si>
+  <si>
+    <t>0909000001</t>
+  </si>
+  <si>
+    <t>Đang làm việc</t>
+  </si>
+  <si>
+    <t>12/12/2025</t>
   </si>
   <si>
     <t>Trần</t>
   </si>
   <si>
-    <t>Trần s</t>
+    <t>Trần Bình</t>
   </si>
   <si>
     <t>0909000002</t>
   </si>
   <si>
+    <t>Trống lịch</t>
+  </si>
+  <si>
     <t>Lê</t>
   </si>
   <si>
@@ -88,12 +91,6 @@
     <t>Lê Cường</t>
   </si>
   <si>
-    <t>0909003003</t>
-  </si>
-  <si>
-    <t>Trống</t>
-  </si>
-  <si>
     <t>Phạm</t>
   </si>
   <si>
@@ -116,6 +113,15 @@
   </si>
   <si>
     <t>0909000005</t>
+  </si>
+  <si>
+    <t>Trân</t>
+  </si>
+  <si>
+    <t>0909003333</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
   <si>
     <t>5</t>
@@ -128,7 +134,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -165,12 +171,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -199,39 +205,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -283,7 +289,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -394,6 +400,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -402,13 +415,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -473,31 +479,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -506,19 +492,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="3" width="9.109375" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" customWidth="1"/>
-    <col min="10" max="10" width="9.109375" customWidth="1"/>
+    <col min="1" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,7 +535,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -570,7 +555,7 @@
         <v>14</v>
       </c>
       <c r="G2" s="3">
-        <v>45566</v>
+        <v>45301</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>15</v>
@@ -582,7 +567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -590,7 +575,7 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
         <v>17</v>
@@ -599,14 +584,12 @@
         <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G3" s="3">
-        <v>45414</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>15</v>
-      </c>
+        <v>45327</v>
+      </c>
+      <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
         <v>15</v>
       </c>
@@ -614,63 +597,59 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G4" s="3">
-        <v>45566</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="2">
-        <v>3</v>
+        <v>45708</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3">
+        <v>46003</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G5" s="3">
-        <v>45294</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>15</v>
-      </c>
+        <v>45352</v>
+      </c>
+      <c r="H5" s="3"/>
       <c r="I5" s="3" t="s">
         <v>15</v>
       </c>
@@ -678,36 +657,34 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>5</v>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G6" s="3">
         <v>45366</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="H6" s="3"/>
       <c r="I6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>32</v>
+      <c r="J6" s="2">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>